<commit_message>
Fix vercel.json: remove duplicate functions property
</commit_message>
<xml_diff>
--- a/SF9 FINAL FORMAT-FRONT.xlsx
+++ b/SF9 FINAL FORMAT-FRONT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedro\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CS_PROJECTS\PGCHSPROGRAMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5485F6AA-5601-4FF4-93A2-30BA87F9D63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F122DEA-F4F4-4882-883B-B4037E9BE7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{83477122-C2C2-4432-940F-079E405C6F8A}"/>
   </bookViews>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="53">
   <si>
     <t>Republika ng Pilipinas</t>
   </si>
@@ -129,12 +120,6 @@
     <t>Technology and Livelihood Education (Creative Tech)</t>
   </si>
   <si>
-    <t xml:space="preserve">         Physical Education and Health</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        Physical Education and Health</t>
-  </si>
-  <si>
     <t>MATHEMATICAL INVESTIGATION AND MODELLING</t>
   </si>
   <si>
@@ -196,6 +181,9 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       Physical Education and Health</t>
   </si>
 </sst>
 </file>
@@ -479,7 +467,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -531,10 +519,95 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -543,97 +616,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1174,193 +1157,193 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="K2" s="32" t="s">
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="K2" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
     </row>
     <row r="3" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="K3" s="32" t="s">
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="K3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="62"/>
+      <c r="Q3" s="62"/>
     </row>
     <row r="4" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="K4" s="32" t="s">
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+      <c r="K4" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="32"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="62"/>
+      <c r="P4" s="62"/>
+      <c r="Q4" s="62"/>
     </row>
     <row r="5" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="K5" s="33" t="s">
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="K5" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
+      <c r="L5" s="60"/>
+      <c r="M5" s="60"/>
+      <c r="N5" s="60"/>
+      <c r="O5" s="60"/>
+      <c r="P5" s="60"/>
+      <c r="Q5" s="60"/>
     </row>
     <row r="6" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="K6" s="34" t="s">
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="61"/>
+      <c r="K6" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="34"/>
-      <c r="Q6" s="34"/>
+      <c r="L6" s="61"/>
+      <c r="M6" s="61"/>
+      <c r="N6" s="61"/>
+      <c r="O6" s="61"/>
+      <c r="P6" s="61"/>
+      <c r="Q6" s="61"/>
     </row>
     <row r="7" spans="2:17" s="1" customFormat="1" ht="12.75">
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="K7" s="32" t="s">
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="K7" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="32"/>
-      <c r="Q7" s="32"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="62"/>
+      <c r="N7" s="62"/>
+      <c r="O7" s="62"/>
+      <c r="P7" s="62"/>
+      <c r="Q7" s="62"/>
     </row>
     <row r="8" spans="2:17" ht="6" customHeight="1"/>
     <row r="9" spans="2:17">
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="K9" s="37" t="s">
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="K9" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="59"/>
+      <c r="P9" s="59"/>
+      <c r="Q9" s="59"/>
     </row>
     <row r="10" spans="2:17" ht="8.25" customHeight="1">
       <c r="B10" s="3"/>
       <c r="K10" s="3"/>
     </row>
     <row r="11" spans="2:17" ht="15.75">
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="38"/>
-      <c r="H11" s="38"/>
-      <c r="K11" s="38" t="s">
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="K11" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="L11" s="38"/>
-      <c r="M11" s="38"/>
-      <c r="N11" s="38"/>
-      <c r="O11" s="38"/>
-      <c r="P11" s="38"/>
-      <c r="Q11" s="38"/>
+      <c r="L11" s="52"/>
+      <c r="M11" s="52"/>
+      <c r="N11" s="52"/>
+      <c r="O11" s="52"/>
+      <c r="P11" s="52"/>
+      <c r="Q11" s="52"/>
     </row>
     <row r="12" spans="2:17">
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="K12" s="35" t="s">
+      <c r="C12" s="58"/>
+      <c r="D12" s="53"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="53"/>
+      <c r="K12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="L12" s="35"/>
-      <c r="M12" s="36"/>
-      <c r="N12" s="36"/>
-      <c r="O12" s="36"/>
+      <c r="L12" s="58"/>
+      <c r="M12" s="53"/>
+      <c r="N12" s="53"/>
+      <c r="O12" s="53"/>
     </row>
     <row r="13" spans="2:17" ht="6.75" customHeight="1"/>
     <row r="14" spans="2:17">
       <c r="B14" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
       <c r="E14" t="s">
         <v>10</v>
       </c>
@@ -1372,8 +1355,8 @@
       <c r="K14" t="s">
         <v>9</v>
       </c>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
+      <c r="L14" s="53"/>
+      <c r="M14" s="53"/>
       <c r="N14" t="s">
         <v>10</v>
       </c>
@@ -1408,7 +1391,7 @@
       <c r="Q15" s="20"/>
     </row>
     <row r="16" spans="2:17">
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="29" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="21"/>
@@ -1417,7 +1400,7 @@
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
       <c r="H16" s="22"/>
-      <c r="K16" s="31" t="s">
+      <c r="K16" s="29" t="s">
         <v>15</v>
       </c>
       <c r="L16" s="21"/>
@@ -1429,18 +1412,18 @@
     </row>
     <row r="17" spans="2:17" ht="11.25" customHeight="1">
       <c r="B17" s="23"/>
-      <c r="C17" s="43" t="s">
+      <c r="C17" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="55"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="23"/>
-      <c r="L17" s="29" t="s">
+      <c r="L17" s="24" t="s">
         <v>16</v>
       </c>
       <c r="M17" s="24"/>
@@ -1450,18 +1433,18 @@
       <c r="Q17" s="25"/>
     </row>
     <row r="18" spans="2:17" ht="11.25" customHeight="1">
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="55"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="30" t="s">
+      <c r="K18" s="23" t="s">
         <v>17</v>
       </c>
       <c r="L18" s="24"/>
@@ -1472,10 +1455,10 @@
       <c r="Q18" s="25"/>
     </row>
     <row r="19" spans="2:17" ht="10.5" customHeight="1">
-      <c r="B19" s="46" t="s">
+      <c r="B19" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="47"/>
+      <c r="C19" s="57"/>
       <c r="D19" s="27"/>
       <c r="E19" s="27"/>
       <c r="F19" s="27"/>
@@ -1493,60 +1476,60 @@
     </row>
     <row r="20" spans="2:17" hidden="1"/>
     <row r="21" spans="2:17" ht="15.75">
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="K21" s="38" t="s">
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="K21" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="L21" s="38"/>
-      <c r="M21" s="38"/>
-      <c r="N21" s="38"/>
-      <c r="O21" s="38"/>
-      <c r="P21" s="38"/>
-      <c r="Q21" s="38"/>
+      <c r="L21" s="52"/>
+      <c r="M21" s="52"/>
+      <c r="N21" s="52"/>
+      <c r="O21" s="52"/>
+      <c r="P21" s="52"/>
+      <c r="Q21" s="52"/>
     </row>
     <row r="22" spans="2:17">
-      <c r="B22" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="50"/>
-      <c r="D22" s="39" t="s">
+      <c r="B22" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="33"/>
+      <c r="D22" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="E22" s="39"/>
-      <c r="F22" s="40"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="49"/>
       <c r="G22" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H22" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="K22" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="H22" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="K22" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="L22" s="50"/>
-      <c r="M22" s="39" t="s">
+      <c r="L22" s="33"/>
+      <c r="M22" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="N22" s="39"/>
-      <c r="O22" s="40"/>
+      <c r="N22" s="48"/>
+      <c r="O22" s="49"/>
       <c r="P22" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q22" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="Q22" s="50" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="2:17">
-      <c r="B23" s="50"/>
-      <c r="C23" s="50"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="33"/>
       <c r="D23" s="6">
         <v>1</v>
       </c>
@@ -1557,11 +1540,11 @@
         <v>3</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H23" s="42"/>
-      <c r="K23" s="50"/>
-      <c r="L23" s="50"/>
+        <v>42</v>
+      </c>
+      <c r="H23" s="51"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
       <c r="M23" s="6">
         <v>1</v>
       </c>
@@ -1572,24 +1555,24 @@
         <v>3</v>
       </c>
       <c r="P23" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q23" s="42"/>
+        <v>42</v>
+      </c>
+      <c r="Q23" s="51"/>
     </row>
     <row r="24" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B24" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="49"/>
+      <c r="B24" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="38"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
       <c r="G24" s="10"/>
       <c r="H24" s="9"/>
-      <c r="K24" s="48" t="s">
-        <v>41</v>
-      </c>
-      <c r="L24" s="49"/>
+      <c r="K24" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="L24" s="38"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
@@ -1597,19 +1580,19 @@
       <c r="Q24" s="9"/>
     </row>
     <row r="25" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B25" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="49"/>
+      <c r="B25" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="38"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
-      <c r="K25" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="L25" s="49"/>
+      <c r="K25" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="L25" s="38"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
       <c r="O25" s="9"/>
@@ -1617,19 +1600,19 @@
       <c r="Q25" s="9"/>
     </row>
     <row r="26" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B26" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26" s="49"/>
+      <c r="B26" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="38"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
-      <c r="K26" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="L26" s="49"/>
+      <c r="K26" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="L26" s="38"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
@@ -1637,19 +1620,19 @@
       <c r="Q26" s="9"/>
     </row>
     <row r="27" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B27" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" s="49"/>
+      <c r="B27" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="38"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
-      <c r="K27" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="L27" s="49"/>
+      <c r="K27" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="L27" s="38"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
@@ -1657,19 +1640,19 @@
       <c r="Q27" s="9"/>
     </row>
     <row r="28" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B28" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="49"/>
+      <c r="B28" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="38"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
-      <c r="K28" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="L28" s="49"/>
+      <c r="K28" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="L28" s="38"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9"/>
       <c r="O28" s="9"/>
@@ -1677,19 +1660,19 @@
       <c r="Q28" s="9"/>
     </row>
     <row r="29" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B29" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="C29" s="54"/>
+      <c r="B29" s="46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="47"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
-      <c r="K29" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="L29" s="49"/>
+      <c r="K29" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="L29" s="38"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9"/>
       <c r="O29" s="9"/>
@@ -1697,19 +1680,19 @@
       <c r="Q29" s="9"/>
     </row>
     <row r="30" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B30" s="51" t="s">
+      <c r="B30" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="52"/>
+      <c r="C30" s="45"/>
       <c r="D30" s="13"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
-      <c r="K30" s="51" t="s">
+      <c r="K30" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="L30" s="52"/>
+      <c r="L30" s="45"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
       <c r="O30" s="9"/>
@@ -1718,7 +1701,7 @@
     </row>
     <row r="31" spans="2:17" ht="12.95" customHeight="1">
       <c r="B31" s="14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C31" s="15"/>
       <c r="D31" s="13"/>
@@ -1727,7 +1710,7 @@
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
       <c r="K31" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L31" s="12"/>
       <c r="M31" s="9"/>
@@ -1758,7 +1741,7 @@
     </row>
     <row r="33" spans="2:17" ht="12.95" customHeight="1">
       <c r="B33" s="11" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="9"/>
@@ -1767,7 +1750,7 @@
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
       <c r="K33" s="11" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="L33" s="16"/>
       <c r="M33" s="9"/>
@@ -1797,19 +1780,19 @@
       <c r="Q34" s="9"/>
     </row>
     <row r="35" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B35" s="55" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="56"/>
+      <c r="B35" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="C35" s="40"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
-      <c r="K35" s="55" t="s">
-        <v>33</v>
-      </c>
-      <c r="L35" s="56"/>
+      <c r="K35" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="L35" s="40"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
       <c r="O35" s="9"/>
@@ -1817,15 +1800,15 @@
       <c r="Q35" s="9"/>
     </row>
     <row r="36" spans="2:17" ht="12.95" customHeight="1">
-      <c r="B36" s="48"/>
-      <c r="C36" s="49"/>
+      <c r="B36" s="37"/>
+      <c r="C36" s="38"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
-      <c r="K36" s="48"/>
-      <c r="L36" s="49"/>
+      <c r="K36" s="37"/>
+      <c r="L36" s="38"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
       <c r="O36" s="9"/>
@@ -1833,239 +1816,268 @@
       <c r="Q36" s="9"/>
     </row>
     <row r="37" spans="2:17" s="19" customFormat="1" ht="12.95" customHeight="1">
-      <c r="B37" s="57" t="s">
+      <c r="B37" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="58"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="59"/>
+      <c r="C37" s="42"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="43"/>
       <c r="G37" s="18"/>
       <c r="H37" s="18"/>
-      <c r="K37" s="57" t="s">
+      <c r="K37" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="L37" s="58"/>
-      <c r="M37" s="58"/>
-      <c r="N37" s="58"/>
-      <c r="O37" s="59"/>
+      <c r="L37" s="42"/>
+      <c r="M37" s="42"/>
+      <c r="N37" s="42"/>
+      <c r="O37" s="43"/>
       <c r="P37" s="18"/>
       <c r="Q37" s="18"/>
     </row>
     <row r="38" spans="2:17" ht="22.5" customHeight="1">
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="K38" s="62" t="s">
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="31"/>
+      <c r="K38" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="L38" s="62"/>
-      <c r="M38" s="62"/>
-      <c r="N38" s="62"/>
-      <c r="O38" s="62"/>
-      <c r="P38" s="62"/>
-      <c r="Q38" s="62"/>
+      <c r="L38" s="32"/>
+      <c r="M38" s="32"/>
+      <c r="N38" s="32"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="32"/>
+      <c r="Q38" s="32"/>
     </row>
     <row r="39" spans="2:17" s="17" customFormat="1" ht="12.95" customHeight="1">
-      <c r="B39" s="50" t="s">
-        <v>52</v>
-      </c>
-      <c r="C39" s="50"/>
-      <c r="D39" s="63" t="s">
-        <v>53</v>
-      </c>
-      <c r="E39" s="64"/>
-      <c r="F39" s="65"/>
-      <c r="G39" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="H39" s="50"/>
-      <c r="K39" s="50" t="s">
-        <v>52</v>
-      </c>
-      <c r="L39" s="50"/>
-      <c r="M39" s="63" t="s">
-        <v>53</v>
-      </c>
-      <c r="N39" s="64"/>
-      <c r="O39" s="65"/>
-      <c r="P39" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q39" s="50"/>
+      <c r="B39" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" s="33"/>
+      <c r="D39" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="E39" s="35"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="H39" s="33"/>
+      <c r="K39" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="L39" s="33"/>
+      <c r="M39" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="N39" s="35"/>
+      <c r="O39" s="36"/>
+      <c r="P39" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q39" s="33"/>
     </row>
     <row r="40" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60" t="s">
+      <c r="C40" s="30"/>
+      <c r="D40" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" s="30"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="H40" s="30"/>
+      <c r="K40" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="L40" s="30"/>
+      <c r="M40" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="N40" s="30"/>
+      <c r="O40" s="30"/>
+      <c r="P40" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q40" s="30"/>
+    </row>
+    <row r="41" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
+      <c r="B41" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41" s="30"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="H41" s="30"/>
+      <c r="K41" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="L41" s="30"/>
+      <c r="M41" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="N41" s="30"/>
+      <c r="O41" s="30"/>
+      <c r="P41" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q41" s="30"/>
+    </row>
+    <row r="42" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
+      <c r="B42" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="E40" s="60"/>
-      <c r="F40" s="60"/>
-      <c r="G40" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H40" s="60"/>
-      <c r="K40" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="L40" s="60"/>
-      <c r="M40" s="60" t="s">
+      <c r="E42" s="30"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="H42" s="30"/>
+      <c r="K42" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="L42" s="30"/>
+      <c r="M42" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="N40" s="60"/>
-      <c r="O40" s="60"/>
-      <c r="P40" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q40" s="60"/>
-    </row>
-    <row r="41" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B41" s="60" t="s">
-        <v>26</v>
-      </c>
-      <c r="C41" s="60"/>
-      <c r="D41" s="60" t="s">
+      <c r="N42" s="30"/>
+      <c r="O42" s="30"/>
+      <c r="P42" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q42" s="30"/>
+    </row>
+    <row r="43" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
+      <c r="B43" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="E41" s="60"/>
-      <c r="F41" s="60"/>
-      <c r="G41" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H41" s="60"/>
-      <c r="K41" s="60" t="s">
-        <v>26</v>
-      </c>
-      <c r="L41" s="60"/>
-      <c r="M41" s="60" t="s">
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="H43" s="30"/>
+      <c r="K43" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="L43" s="30"/>
+      <c r="M43" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="N41" s="60"/>
-      <c r="O41" s="60"/>
-      <c r="P41" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q41" s="60"/>
-    </row>
-    <row r="42" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B42" s="60" t="s">
-        <v>27</v>
-      </c>
-      <c r="C42" s="60"/>
-      <c r="D42" s="60" t="s">
+      <c r="N43" s="30"/>
+      <c r="O43" s="30"/>
+      <c r="P43" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q43" s="30"/>
+    </row>
+    <row r="44" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
+      <c r="B44" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="E42" s="60"/>
-      <c r="F42" s="60"/>
-      <c r="G42" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H42" s="60"/>
-      <c r="K42" s="60" t="s">
-        <v>27</v>
-      </c>
-      <c r="L42" s="60"/>
-      <c r="M42" s="60" t="s">
+      <c r="E44" s="30"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="H44" s="30"/>
+      <c r="K44" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="L44" s="30"/>
+      <c r="M44" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="N42" s="60"/>
-      <c r="O42" s="60"/>
-      <c r="P42" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q42" s="60"/>
-    </row>
-    <row r="43" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B43" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C43" s="60"/>
-      <c r="D43" s="60" t="s">
+      <c r="N44" s="30"/>
+      <c r="O44" s="30"/>
+      <c r="P44" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="E43" s="60"/>
-      <c r="F43" s="60"/>
-      <c r="G43" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H43" s="60"/>
-      <c r="K43" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="L43" s="60"/>
-      <c r="M43" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="N43" s="60"/>
-      <c r="O43" s="60"/>
-      <c r="P43" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q43" s="60"/>
-    </row>
-    <row r="44" spans="2:17" s="17" customFormat="1" ht="15" customHeight="1">
-      <c r="B44" s="60" t="s">
-        <v>29</v>
-      </c>
-      <c r="C44" s="60"/>
-      <c r="D44" s="60" t="s">
-        <v>50</v>
-      </c>
-      <c r="E44" s="60"/>
-      <c r="F44" s="60"/>
-      <c r="G44" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H44" s="60"/>
-      <c r="K44" s="60" t="s">
-        <v>29</v>
-      </c>
-      <c r="L44" s="60"/>
-      <c r="M44" s="60" t="s">
-        <v>50</v>
-      </c>
-      <c r="N44" s="60"/>
-      <c r="O44" s="60"/>
-      <c r="P44" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q44" s="60"/>
+      <c r="Q44" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="91">
-    <mergeCell ref="P44:Q44"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="M43:O43"/>
-    <mergeCell ref="P43:Q43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:O44"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="M41:O41"/>
-    <mergeCell ref="P41:Q41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="K42:L42"/>
-    <mergeCell ref="M42:O42"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="K2:Q2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="K3:Q3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="K4:Q4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="K5:Q5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="K7:Q7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="K9:Q9"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="K11:Q11"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="B22:C23"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="K22:L23"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="K37:O37"/>
     <mergeCell ref="P40:Q40"/>
     <mergeCell ref="B38:H38"/>
     <mergeCell ref="K38:Q38"/>
@@ -2080,59 +2092,30 @@
     <mergeCell ref="G40:H40"/>
     <mergeCell ref="K40:L40"/>
     <mergeCell ref="M40:O40"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="K37:O37"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="B22:C23"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="K22:L23"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="Q22:Q23"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="K21:Q21"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="M12:O12"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="K9:Q9"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="K11:Q11"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="K5:Q5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="K7:Q7"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="K2:Q2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="K3:Q3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="K4:Q4"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="M41:O41"/>
+    <mergeCell ref="P41:Q41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="M42:O42"/>
+    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="M43:O43"/>
+    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:O44"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>